<commit_message>
✨ feat(Bench_Ben-Cist1.py): add save_df_as_json_records utility
- refactor file saving logic to use save_df_as_json_records from neddata.utils.fileio
- update pooch registry hash for Bench_Ben-Cist1.json and Bench_Ben-Cist1.xlsx

♻️ refactor(datamodel.py): enhance _write_registry and _clean_registry functions

- add verbose output for removed entries in _write_registry
- return list of removed entries from _clean_registry
- improve readability and formatting

🔧 chore(fileio.py): add save_df_as_json_records function

- implement save_df_as_json_records to save DataFrame as JSON records
</commit_message>
<xml_diff>
--- a/src/neddata/abbey/Benchmark/Bench_Ben-Cist1.xlsx
+++ b/src/neddata/abbey/Benchmark/Bench_Ben-Cist1.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Albertus Greue Graue, Greuen | prov. de can. c. reserv. preb. eccl. s. Johannis Osnaburg. ac benef. ad coll. abb. etc. mon. Corbien. o. s. Ben. Paderburn. dioc., n. o. vicar. ad alt. ss. Marie Magdalene et Barbare in par. eccl. Quakenburgen. Osnaburg. dioc. 27 apr. 1424 L 246 156r.</t>
+          <t>Albertus Greue Graue, Greuen || prov. de can. c. reserv. preb. eccl. s. Johannis Osnaburg. ac benef. ad coll. abb. etc. mon. Corbien. o. s. Ben. Paderburn. dioc., n. o. vicar. ad alt. ss. Marie Magdalene et Barbare in par. eccl. Quakenburgen. Osnaburg. dioc. 27 apr. 1424 L 246 156r.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bartholomeus abb. et monach. mon. s. Laurentii o. s. Ben. e. m. Leod. | inter al. referentes quod Nicolaus V. pro eo quod nonnulli aep. ep. et aliquarum ecclesiarum prelati contra privilegia decanis et capitulis colleg. ecclesiarum civit. et dioc. Leod. conc. eisdem decanis etc. iniurias inferre conabantur litteras dedit in mandatum abbati eccl. s. Laurentii e. m. Leod. et prepositis eccl. ss. Appl. Colon. et eccl. s. Johannis Traiect. ut n. permitterent eos indebite molestari quodque papa iudicibus dedit in mandatum ut contra d. aep. et al. dd. decanis etc. iniurias inferentes providerent: de conserv. 3. mart. 78 S 766 67rss.</t>
+          <t>Bartholomeus abb. et monach. mon. s. Laurentii o. s. Ben. e. m. Leod. || inter al. referentes quod Nicolaus V. pro eo quod nonnulli aep. ep. et aliquarum ecclesiarum prelati contra privilegia decanis et capitulis colleg. ecclesiarum civit. et dioc. Leod. conc. eisdem decanis etc. iniurias inferre conabantur litteras dedit in mandatum abbati eccl. s. Laurentii e. m. Leod. et prepositis eccl. ss. Appl. Colon. et eccl. s. Johannis Traiect. ut n. permitterent eos indebite molestari quodque papa iudicibus dedit in mandatum ut contra d. aep. et al. dd. decanis etc. iniurias inferentes providerent: de conserv. 3. mart. 78 S 766 67rss.</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Castellum | abb. etc. mon. o. s. Ben. Eistet. dioc. : de conf. emptionis grangie in Heburgen d. dioc. a prep. etc. mon. s. Petri in Pertholtzgaden o. s. Aug. Salzeburg. dioc. 31 iul. 1418 S 115 224v, L 247 247r.</t>
+          <t>Castellum || abb. etc. mon. o. s. Ben. Eistet. dioc. : de conf. emptionis grangie in Heburgen d. dioc. a prep. etc. mon. s. Petri in Pertholtzgaden o. s. Aug. Salzeburg. dioc. 31 iul. 1418 S 115 224v, L 247 247r.</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Hartungus Crutzeburg | conf. vicar. ad alt. omn. SS. in eccl. s. Petri Fritzlar. Magunt. dioc. vac. p. o. Bertoldi Israel ei coll. ab Innoc. VII, n. o. benef. ad coll. dec. etc. eccl. b. Marie Isenac. d. dioc., abb. etc. mon. Hersfeld. o. s. Ben. d. dioc., 19 dec. 1406 L 132 108v.</t>
+          <t>Hartungus Crutzeburg || conf. vicar. ad alt. omn. SS. in eccl. s. Petri Fritzlar. Magunt. dioc. vac. p. o. Bertoldi Israel ei coll. ab Innoc. VII, n. o. benef. ad coll. dec. etc. eccl. b. Marie Isenac. d. dioc., abb. etc. mon. Hersfeld. o. s. Ben. d. dioc., 19 dec. 1406 L 132 108v.</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Henricus de Zoemeren presb. Leod. dioc. mag. in theol. | can. eccl. s. Petri Lovanien. Leod. dioc. qui vig. gr. expect. de 2 benef. ad coll. abbatum etc. Epternacen. et Egmonden. o.s. Ben. Trever. et Traiect. dioc. par. eccl. de Eisel Leod. dioc. 15 m. arg. vac. p.o. Arnoldi Baest quond. Nicolai tit. s. Petri ad vincula card. fam. acc.: m. Adriano de Hee can. eccl. Leod. et al. confer. de novo d. par. eccl. 26. apr. 1467 V 536 188r-190r.</t>
+          <t>Henricus de Zoemeren presb. Leod. dioc. mag. in theol. || can. eccl. s. Petri Lovanien. Leod. dioc. qui vig. gr. expect. de 2 benef. ad coll. abbatum etc. Epternacen. et Egmonden. o.s. Ben. Trever. et Traiect. dioc. par. eccl. de Eisel Leod. dioc. 15 m. arg. vac. p.o. Arnoldi Baest quond. Nicolai tit. s. Petri ad vincula card. fam. acc.: m. Adriano de Hee can. eccl. Leod. et al. confer. de novo d. par. eccl. 26. apr. 1467 V 536 188r-190r.</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Johannes Derres cler. Magunt. dioc. | presb. Magunt. dioc.: de nova prov. de par. eccl. in Brampach maior. d. dioc. 4 m. arg. quam vac. p. o. Henrici Cruezbourg Crutzeburg acc. vig. gr. expect. &lt;de 2 benef. ad coll. abb. etc. mon. Hersfelden. o. s. Ben. necnon prep. etc. eccl. s. Petri Fritzlarien. d. dioc.&gt;, n. o. perp. s. c. vicar. ad alt. s. Viti in eccl. s. Petri Fritzlarien. 4 m. arg. litig. in cur. quam n. possidet &lt;c. cass. gr. expect. in casu pacifice possessionis d. eccl.&gt; 18. aug. 1463 S 556 137vs., L 584 268rss.</t>
+          <t>Johannes Derres cler. Magunt. dioc. || presb. Magunt. dioc.: de nova prov. de par. eccl. in Brampach maior. d. dioc. 4 m. arg. quam vac. p. o. Henrici Cruezbourg Crutzeburg acc. vig. gr. expect. &lt;de 2 benef. ad coll. abb. etc. mon. Hersfelden. o. s. Ben. necnon prep. etc. eccl. s. Petri Fritzlarien. d. dioc.&gt;, n. o. perp. s. c. vicar. ad alt. s. Viti in eccl. s. Petri Fritzlarien. 4 m. arg. litig. in cur. quam n. possidet &lt;c. cass. gr. expect. in casu pacifice possessionis d. eccl.&gt; 18. aug. 1463 S 556 137vs., L 584 268rss.</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Johannes Mentzer de Huchelnheim presb. Magunt. bac. in art. | f. gr. de benef. ad coll. abb. etc. mon. Fulden., prep. etc. mon. Montissanctipetri prope Fuldam o. s. Ben. Herbip. dioc., n. o. benef. ad coll. prep. etc. eccl. s. Stephani Magunt. dioc. dim. quoad cur., 15 sept. 1397 L 49 279.</t>
+          <t>Johannes Mentzer de Huchelnheim presb. Magunt. bac. in art. || f. gr. de benef. ad coll. abb. etc. mon. Fulden., prep. etc. mon. Montissanctipetri prope Fuldam o. s. Ben. Herbip. dioc., n. o. benef. ad coll. prep. etc. eccl. s. Stephani Magunt. dioc. dim. quoad cur., 15 sept. 1397 L 49 279.</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Johannes Neve (Nepos, New, Neeff) cler. Leod. dioc. | pape fam. qui vig. gr. expect. sibi s. d. 1. ian. 72 de 2 benef. ad coll. abba. et conv. mon. s. Salvatoris in Susteren o. s. Ben. Leod. dioc. ac ad coll. prep. prepos. in Mersem o. s. Ben. Leod. dioc. conc. par. eccl. de Mersen Leod. dioc. ad coll. d. prep. acc. quam n. possidet et sup. qua litig. in cur. contra quendam adversarium: de cass. dd. litt. quoad coll. dd. abba. etc. et de decl. dd. litt. perinde val. acsi p. priores litt. de can. et preb. eccl. s. Gereonis Colon. necnon de benef. ad coll. ep. etc. Traiect. prov. fuisset sub dim. d. par. eccl., gratis 7. iun. 75 V 678 648r -650v</t>
+          <t>Johannes Neve (Nepos, New, Neeff) cler. Leod. dioc. || pape fam. qui vig. gr. expect. sibi s. d. 1. ian. 72 de 2 benef. ad coll. abba. et conv. mon. s. Salvatoris in Susteren o. s. Ben. Leod. dioc. ac ad coll. prep. prepos. in Mersem o. s. Ben. Leod. dioc. conc. par. eccl. de Mersen Leod. dioc. ad coll. d. prep. acc. quam n. possidet et sup. qua litig. in cur. contra quendam adversarium: de cass. dd. litt. quoad coll. dd. abba. etc. et de decl. dd. litt. perinde val. acsi p. priores litt. de can. et preb. eccl. s. Gereonis Colon. necnon de benef. ad coll. ep. etc. Traiect. prov. fuisset sub dim. d. par. eccl., gratis 7. iun. 75 V 678 648r -650v</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Johannes Prumer (Pruner, Prunner) pape fam. | gr. expect. de can. et preb. eccl. s. Swiberti in Werdena (Verdena) Principis [= Kaiserswerth] Colon. dioc. necnon de benef. ad coll. abba. etc. mon. Valliscomitis o. Cist. Colon. dioc. (exec. ep. Vasionen. et dec. eccl. s. Victoris Xancten. Colon. dioc. et dec. eccl. s. Martini Embricen. Traiect. dioc.), gratis 20. apr. 75 V 664 248r -250v</t>
+          <t>Johannes Prumer (Pruner, Prunner) pape fam. || gr. expect. de can. et preb. eccl. s. Swiberti in Werdena (Verdena) Principis [= Kaiserswerth] Colon. dioc. necnon de benef. ad coll. abba. etc. mon. Valliscomitis o. Cist. Colon. dioc. (exec. ep. Vasionen. et dec. eccl. s. Victoris Xancten. Colon. dioc. et dec. eccl. s. Martini Embricen. Traiect. dioc.), gratis 20. apr. 75 V 664 248r -250v</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Johannes Vrese cler. Traiect. dioc. | prov. de can. eccl. s. Lebuini Daventrien. Traiect. dioc. c. reserv. preb. et dign. necnon de benef. ad coll. abb. etc. mon. s. Adelberti Egmond. o. s. Ben. d. dioc. 20 apr. 1455 L 499 152v-154v.</t>
+          <t>Johannes Vrese cler. Traiect. dioc. || prov. de can. eccl. s. Lebuini Daventrien. Traiect. dioc. c. reserv. preb. et dign. necnon de benef. ad coll. abb. etc. mon. s. Adelberti Egmond. o. s. Ben. d. dioc. 20 apr. 1455 L 499 152v-154v.</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Johannes Waydenhofel cler. Ratisbon. dioc. | cui gr. expect. s. d. 1. ian. 72 de 2 benef. ad coll. mon. s. Emerami Ratisbon. dioc. o. s. Ben. et mon. in Waldsachssen o. Cist. Ratisbon. dioc. conc. fuit: de decl. litt. desup. perinde val. acsi temp. d. gr. expect. pape fam. fuisset 4. iun. 73 S 691 166rs.</t>
+          <t>Johannes Waydenhofel cler. Ratisbon. dioc. || cui gr. expect. s. d. 1. ian. 72 de 2 benef. ad coll. mon. s. Emerami Ratisbon. dioc. o. s. Ben. et mon. in Waldsachssen o. Cist. Ratisbon. dioc. conc. fuit: de decl. litt. desup. perinde val. acsi temp. d. gr. expect. pape fam. fuisset 4. iun. 73 S 691 166rs.</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Johannes de Ortemberg Ortenberg, qui prov. est s. d. 17 mart. 13 post resign. Johannis Potis | cler. Trever. dioc. cum disp. super def. nat.: m. prov. super can. et preb. mon. in Dytkirchen e. m. Bunnen. o. s. Ben. et vic. par. eccl. s. Remigii Bunnen. Colon. dioc. vac. per resign. Theoderici de Broech coram Frederico aep. Colon., n. o. prov. super vic. s. Barbare in eccl. ss. apl. Colon. ac s. Trinitatis in eccl. s. Cassii Bunnen. Colon. dioc. 20 oct. 1413 L 170 137.</t>
+          <t>Johannes de Ortemberg Ortenberg, qui prov. est s. d. 17 mart. 13 post resign. Johannis Potis || cler. Trever. dioc. cum disp. super def. nat.: m. prov. super can. et preb. mon. in Dytkirchen e. m. Bunnen. o. s. Ben. et vic. par. eccl. s. Remigii Bunnen. Colon. dioc. vac. per resign. Theoderici de Broech coram Frederico aep. Colon., n. o. prov. super vic. s. Barbare in eccl. ss. apl. Colon. ac s. Trinitatis in eccl. s. Cassii Bunnen. Colon. dioc. 20 oct. 1413 L 170 137.</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Lucas Mitterperger presb. Salzeburg. dioc. | cler. &lt;presb.&gt; Salzeburg. dioc., qui ad par. eccl. s. Michaelis prope Liesinck d. dioc. 6 m. arg. vac. p.o. cuiusdam Stephani p. Andream [de Stetthaim] abb. etc. mon. Admonten. o. s. Ben. d. dioc. ad quos present. de consuetudine pertin. Johanni [de Reisberg] aep. Salzeburg. present. est et eam absque instit. ordin. apprehendit, dim.: nova prov. de d. par. eccl. vac. p.o. Nicolai Raed 24. apr. 37 exec.: ep. Seccov., abb. mon. Admonten. Salzeburg. dioc. et dec. eccl. b. Marie Traiect. exped. 27. apr. 37 L 353 72rss, disp. sup. inhabil. 24. apr. 37 L 353 71vs, l. duarum b. apr. 37 T 5 71r, o.s.a. 3. mai. 37 A 7 82r, solv. personaliter 11 fl. pro compositione ann. 3. mai. 1437 IE 399 53r, IE 400 54r.</t>
+          <t>Lucas Mitterperger presb. Salzeburg. dioc. || cler. &lt;presb.&gt; Salzeburg. dioc., qui ad par. eccl. s. Michaelis prope Liesinck d. dioc. 6 m. arg. vac. p.o. cuiusdam Stephani p. Andream [de Stetthaim] abb. etc. mon. Admonten. o. s. Ben. d. dioc. ad quos present. de consuetudine pertin. Johanni [de Reisberg] aep. Salzeburg. present. est et eam absque instit. ordin. apprehendit, dim.: nova prov. de d. par. eccl. vac. p.o. Nicolai Raed 24. apr. 37 exec.: ep. Seccov., abb. mon. Admonten. Salzeburg. dioc. et dec. eccl. b. Marie Traiect. exped. 27. apr. 37 L 353 72rss, disp. sup. inhabil. 24. apr. 37 L 353 71vs, l. duarum b. apr. 37 T 5 71r, o.s.a. 3. mai. 37 A 7 82r, solv. personaliter 11 fl. pro compositione ann. 3. mai. 1437 IE 399 53r, IE 400 54r.</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Munichszaurach Abb. et conv. mon. in Munichszaurach (Munchawrach) o. s. Ben. Herbip. dioc. cui par. eccl. in Emszkirchen (Empszkirchen) Herbip. dioc. (15 m. arg.) p. Calixtum III. unita fuit et litig. coram certo delegato tunc legato de latere in partibus | referentes quod quond. Johannes [de Grumbach] ep. Herbip. et prep. eccl. s. Gumperti in Onolspach Herbip. dioc. vig. litt. p. Calixtum III. conc. par. eccl. s. Kiliani in Emszkirchen Herbip. dioc. que d. mon. contigua exist. et cuius rectoris present. ad d. mon. pertin. (16 m. arg.) vac. p. o. Reynhardi Speth motu pr. incorp. et quod ipsi desup. litig. vig. commiss. p. Franciscum [Todeschini-Piccolomini] tit. s. Eustachii diac. card. Senen. tunc in illis partibus legatum de latere fact. coram Henrico Furrer dec. eccl. s. Johannis in Haugis e. m. Herbip. et coram Antonio de Grassis aud. contra quond. Georgium Clawbenpusch cler. et coram Johanne Francisco de Pavinis aud. contra Johannem Kraenfues cler. ac quod d. Johannes Kraenfues pro complemento concordie in manibus Jodoci Bellinger (Pewinger) laic. August. dioc. not. publ. resign.: de decl. litt. desup. perinde val. acsi litt. d. unionis plenam firmitatem roboris obtin. etiam si d. par. eccl. vac. p. resign. d. Georgi conc. fuisset 18. apr. 81 S 801 21r , V 610 27r-30r</t>
+          <t>Munichszaurach Abb. et conv. mon. in Munichszaurach (Munchawrach) o. s. Ben. Herbip. dioc. cui par. eccl. in Emszkirchen (Empszkirchen) Herbip. dioc. (15 m. arg.) p. Calixtum III. unita fuit et litig. coram certo delegato tunc legato de latere in partibus || referentes quod quond. Johannes [de Grumbach] ep. Herbip. et prep. eccl. s. Gumperti in Onolspach Herbip. dioc. vig. litt. p. Calixtum III. conc. par. eccl. s. Kiliani in Emszkirchen Herbip. dioc. que d. mon. contigua exist. et cuius rectoris present. ad d. mon. pertin. (16 m. arg.) vac. p. o. Reynhardi Speth motu pr. incorp. et quod ipsi desup. litig. vig. commiss. p. Franciscum [Todeschini-Piccolomini] tit. s. Eustachii diac. card. Senen. tunc in illis partibus legatum de latere fact. coram Henrico Furrer dec. eccl. s. Johannis in Haugis e. m. Herbip. et coram Antonio de Grassis aud. contra quond. Georgium Clawbenpusch cler. et coram Johanne Francisco de Pavinis aud. contra Johannem Kraenfues cler. ac quod d. Johannes Kraenfues pro complemento concordie in manibus Jodoci Bellinger (Pewinger) laic. August. dioc. not. publ. resign.: de decl. litt. desup. perinde val. acsi litt. d. unionis plenam firmitatem roboris obtin. etiam si d. par. eccl. vac. p. resign. d. Georgi conc. fuisset 18. apr. 81 S 801 21r , V 610 27r-30r</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Nicolaus Carnificis cler. Trever. dioc. qui ad par. eccl. s. Albani in Exwiler Trever. dioc. vac. p. o. Henrici Reppynys (Kyppenys) p. abb. mon. s. Mauritii de Tulley o. s. Ben. Trever. dioc. present. et p. archid. de Tulley Trever. dioc. instit. fuit | de nova prov. de d. par. eccl. (6 m. arg.) 25. nov. 78 S 780 90r , m. (dec. eccl. s. Paulini e. m. Trever.) (exped. 24. apr. 79) L 791 204rss.</t>
+          <t>Nicolaus Carnificis cler. Trever. dioc. qui ad par. eccl. s. Albani in Exwiler Trever. dioc. vac. p. o. Henrici Reppynys (Kyppenys) p. abb. mon. s. Mauritii de Tulley o. s. Ben. Trever. dioc. present. et p. archid. de Tulley Trever. dioc. instit. fuit || de nova prov. de d. par. eccl. (6 m. arg.) 25. nov. 78 S 780 90r , m. (dec. eccl. s. Paulini e. m. Trever.) (exped. 24. apr. 79) L 791 204rss.</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Nicolaus Gundelfinger Nicolaus Gundelfinger Gundefingen, Sundelsinger, Sundersinger cler. Constant. dioc., licent. in decr. | de perinde valere prov. de can. et preb. eccl. Constant. 16 m. arg. ; n.o. disp. sup. def. nat. acol. o. s. Ben., s. 12. febr. 1433 S 284 56v.</t>
+          <t>Nicolaus Gundelfinger Nicolaus Gundelfinger Gundefingen, Sundelsinger, Sundersinger cler. Constant. dioc., licent. in decr. || de perinde valere prov. de can. et preb. eccl. Constant. 16 m. arg. ; n.o. disp. sup. def. nat. acol. o. s. Ben., s. 12. febr. 1433 S 284 56v.</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Schonaw | Abb. etc. mon. in S. o. Cist. Wormat. dioc. qui de scitu Petri tit. s. Vitalis presb. card. qui eccl. August. preest vendiderunt abbati etc. mon. in Elwangen o. s. Ben. August. dioc. quandam decimam bladorum et vini op. Schrieshem Wormat. dioc. : m. approb. 11. aug. 1459 L 543 176rs.</t>
+          <t>Schonaw || Abb. etc. mon. in S. o. Cist. Wormat. dioc. qui de scitu Petri tit. s. Vitalis presb. card. qui eccl. August. preest vendiderunt abbati etc. mon. in Elwangen o. s. Ben. August. dioc. quandam decimam bladorum et vini op. Schrieshem Wormat. dioc. : m. approb. 11. aug. 1459 L 543 176rs.</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Thomas Dionisii pape fam. | motu pr. gr. expect. s. d. 1. ian. 72 de can. et preb. eccl. s. Johannis Leod. necnon de benef. ad coll. abb. etc. mon. s. Trudonis de Sancto Trudone o. s. Ben. Leod. dioc. et prerog. ad instar pape fam. descript. (m. Michaeli Moner can. eccl. Elnen. et officialibus Leod. ac Traiect.), gratis 13. mai. 79 V 672 129v -132r</t>
+          <t>Thomas Dionisii pape fam. || motu pr. gr. expect. s. d. 1. ian. 72 de can. et preb. eccl. s. Johannis Leod. necnon de benef. ad coll. abb. etc. mon. s. Trudonis de Sancto Trudone o. s. Ben. Leod. dioc. et prerog. ad instar pape fam. descript. (m. Michaeli Moner can. eccl. Elnen. et officialibus Leod. ac Traiect.), gratis 13. mai. 79 V 672 129v -132r</t>
         </is>
       </c>
     </row>
@@ -964,7 +964,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Thorna Abba. et conv. mon. b. Marie Tho- ren. o. s. Ben. Leod. dioc. | de conf. fundationem et consuetudines d. mon. sup. coll. et recept. abba. et can. 24. decb. 77 S 762 285rs, (m. decanis eccl. s. Andree Colon. et eccl. s. Pauli Leod. ac eccl. s. Servatii Traiecten. Leod. dioc.) L 778 84v - 86r</t>
+          <t>Thorna Abba. et conv. mon. b. Marie Tho- ren. o. s. Ben. Leod. dioc. || de conf. fundationem et consuetudines d. mon. sup. coll. et recept. abba. et can. 24. decb. 77 S 762 285rs, (m. decanis eccl. s. Andree Colon. et eccl. s. Pauli Leod. ac eccl. s. Servatii Traiecten. Leod. dioc.) L 778 84v - 86r</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>fr. Johannes Ruysch Kunsch, Wsch monach. mon. s. Laurentii in Oesbrock Oesbroeck e.m. Traiect. o. s. Ben., &lt;presb.&gt; | preficitur d. mon. vac. p.o. Johannis de Wlne abb. 12. iun. 33 OS 66 25v, solite litt. Florenz, Magl. Classe XXXI, 63 29r, solv. 56 fl. 12 sol. 6 den. pro commun. et min. serv. &lt;50 fl. pro commun. serv. et 6 fl. 12 sol. 6 den. pro min. serv. p.m. Henrici Vos can. eccl. s. Johannis Traiect.&gt; 20. iun. 33 OS 63 245v, 23. iun. 33 Q 1118 110r, oblig. p. d. H. V. 23. iun. 33 OS 64 173v, OS 70 87r, solv. 50 fl. pro commun. serv. 23. iun. 33 IE 394 48r, IE 395 3r, IE 396 2r, solv. 56 fl. 12 sol. 6 den. 26. iun. 33 OS 65 187v, solv. 6 fl. 12 sol. 6 den. pro min. serv. iun. 33 SM 2 7r, solv. 5 fl. pro sacris iun. 33 SM 2 34r, solv. 1 fl. pro sigillo quitantie iun. 33 SM 2 66v, solv. 1 fl. 33 sol. 4 den. pro subdiacon. iun. 1433 SM 2 137r.</t>
+          <t>fr. Johannes Ruysch Kunsch, Wsch monach. mon. s. Laurentii in Oesbrock Oesbroeck e.m. Traiect. o. s. Ben., &lt;presb.&gt; || preficitur d. mon. vac. p.o. Johannis de Wlne abb. 12. iun. 33 OS 66 25v, solite litt. Florenz, Magl. Classe XXXI, 63 29r, solv. 56 fl. 12 sol. 6 den. pro commun. et min. serv. &lt;50 fl. pro commun. serv. et 6 fl. 12 sol. 6 den. pro min. serv. p.m. Henrici Vos can. eccl. s. Johannis Traiect.&gt; 20. iun. 33 OS 63 245v, 23. iun. 33 Q 1118 110r, oblig. p. d. H. V. 23. iun. 33 OS 64 173v, OS 70 87r, solv. 50 fl. pro commun. serv. 23. iun. 33 IE 394 48r, IE 395 3r, IE 396 2r, solv. 56 fl. 12 sol. 6 den. 26. iun. 33 OS 65 187v, solv. 6 fl. 12 sol. 6 den. pro min. serv. iun. 33 SM 2 7r, solv. 5 fl. pro sacris iun. 33 SM 2 34r, solv. 1 fl. pro sigillo quitantie iun. 33 SM 2 66v, solv. 1 fl. 33 sol. 4 den. pro subdiacon. iun. 1433 SM 2 137r.</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Diethelmus monach. mon. s. Gregorii in Petridomo e. m. Constant. o. s. Ben. | oblig. p. Nicolaum Marschalk can. eccl. s. Johannis Constant. 3 dec. 1427 OC 3 207r.</t>
+          <t>Diethelmus monach. mon. s. Gregorii in Petridomo e. m. Constant. o. s. Ben. || oblig. p. Nicolaum Marschalk can. eccl. s. Johannis Constant. 3 dec. 1427 OC 3 207r.</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Gerardus Lausynck de Monte cler. Traiect. dioc. | referens quod Johannes de Monte cler. Traiect. dioc. vig. gr. expect. de can. et preb. eccl. b. Marie in Capitolio Colon. necnon de benef. ad coll. abb. etc. mon. in Siberg o. s. Ben. Colon. dioc. conc. par. eccl. de Oeverrode Colon. dioc. vac. p. o. Sibelionis de Langescheyt acc. et litig. desup. primo coram Nicolao de Edam et secundo coram Bartholomeo de Bellencinis auditoribus et tertio coram Johanne [de Ceretanis] ep. Nucerin. aud. locumtenenti contra quond. Laurentium Rindorp pape fam. et post eius o. in cur. de d. par. eccl. s. d. 3. oct. 77 sibi prov. fuit (litt. n. confectis) et postremo resign. in manibus pape (p. Johannem de Heesbom prep. eccl. s. Andree Colon. procur. fact.): m. (prep. eccl. s. Georgii Colon.) confer. d. par. eccl. (4 m. arg. p.) 15. apr. 79 (exped. 22. apr. 79) L 793 197r -199r.</t>
+          <t>Gerardus Lausynck de Monte cler. Traiect. dioc. || referens quod Johannes de Monte cler. Traiect. dioc. vig. gr. expect. de can. et preb. eccl. b. Marie in Capitolio Colon. necnon de benef. ad coll. abb. etc. mon. in Siberg o. s. Ben. Colon. dioc. conc. par. eccl. de Oeverrode Colon. dioc. vac. p. o. Sibelionis de Langescheyt acc. et litig. desup. primo coram Nicolao de Edam et secundo coram Bartholomeo de Bellencinis auditoribus et tertio coram Johanne [de Ceretanis] ep. Nucerin. aud. locumtenenti contra quond. Laurentium Rindorp pape fam. et post eius o. in cur. de d. par. eccl. s. d. 3. oct. 77 sibi prov. fuit (litt. n. confectis) et postremo resign. in manibus pape (p. Johannem de Heesbom prep. eccl. s. Andree Colon. procur. fact.): m. (prep. eccl. s. Georgii Colon.) confer. d. par. eccl. (4 m. arg. p.) 15. apr. 79 (exped. 22. apr. 79) L 793 197r -199r.</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Henricus Henrici de Cochme cler. Trever. | de vicar. ad alt. omn. SS. in eccl. mon. s. Mathie e. m. Trever. o. s. Ben. vacat. p. ingr. Johannis Franck in d. o. 20 oct. 1419 S 133 187.</t>
+          <t>Henricus Henrici de Cochme cler. Trever. || de vicar. ad alt. omn. SS. in eccl. mon. s. Mathie e. m. Trever. o. s. Ben. vacat. p. ingr. Johannis Franck in d. o. 20 oct. 1419 S 133 187.</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Henricus Knippinch | abb. mon. ss. Petri et Pauli Paderburn. o. s. Ben.: oblig. p. Hartungum Molitoris de Cappel 16 febr. 1405 O 57 123v et Q 48.</t>
+          <t>Henricus Knippinch || abb. mon. ss. Petri et Pauli Paderburn. o. s. Ben.: oblig. p. Hartungum Molitoris de Cappel 16 febr. 1405 O 57 123v et Q 48.</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Johannes Wydenroyd Johannes Wydenroyd Wydenrod, Wideroide cler. Colon., qui vig. surrog. ad iur. alicuius nunc defuncti can. et preb. mon. in Vilich o. s. Ben. Colon. dioc. et par. eccl. de V. insimul 6 m. arg. acc. | de can. et preb. eccl. Traiect. 16 m. arg. vac. p. resign. Cunczonis [de Zwolla] ep. Olomuc.; n.o. can. et preb. eccl. ss. Crisanti et Darie Monasterii Eyflie 8 m. arg. , prov. de can. et preb. eccl. mon. in Vilich o. s. Ben. Colon. dioc. quib. par. eccl. seu pleban. annexa est 6 m. arg. et prov. de vicar. sco[lasti]ci nunc. in eccl. Prag. 8 m. arg. 17. decb. 1431 S 273 92rs.</t>
+          <t>Johannes Wydenroyd Johannes Wydenroyd Wydenrod, Wideroide cler. Colon., qui vig. surrog. ad iur. alicuius nunc defuncti can. et preb. mon. in Vilich o. s. Ben. Colon. dioc. et par. eccl. de V. insimul 6 m. arg. acc. || de can. et preb. eccl. Traiect. 16 m. arg. vac. p. resign. Cunczonis [de Zwolla] ep. Olomuc.; n.o. can. et preb. eccl. ss. Crisanti et Darie Monasterii Eyflie 8 m. arg. , prov. de can. et preb. eccl. mon. in Vilich o. s. Ben. Colon. dioc. quib. par. eccl. seu pleban. annexa est 6 m. arg. et prov. de vicar. sco[lasti]ci nunc. in eccl. Prag. 8 m. arg. 17. decb. 1431 S 273 92rs.</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Johannes [de Werdenberg] ep. August. | et presidentes o. s. Ben. inter al. referentes quod Udalricus Huser, Wilhelmus Stendlin, Jodocus Stetter, Udalricus Harder, Lucas Lanczherre, Johannes Brey et Bartholomeus Kystner monachi mon. ss. Alexandri et Theodori mart. in Ottenbeuren o. s. Ben. reg. observ. August. dioc. e d. mon. exierunt ac mitram baculum et al. bona asportarunt et vitam vagabundam ducebant quodque d. ep. et Wilhelmus [de Lustenau] abb. d. mon. in Ottenbeuren litig. contra dd. monachos coram Udalrico [RÃ¶sch] abb. mon. s. Galli de Sancto Gallo Constant. dioc. et coram quond. Johanne de Cesarinis aud. quodque d. ep. d. Wilhelmum propter delapidationem bonorum et al. excessus aliquamdiu suspendit quodque causa abbatibus d. mon. s. Galli et mon. in Salmansweiler Constant. dioc. et deinde Johanni [de Ceretanis] ep. Nucerin. aud. locumtenenti et deinde Johanni Francisco de Pavinis aud. et postremo magistro Johanni de Duchis prep. eccl. Brixien. utr. iur. doct. pape not. commissa fuit: motu pr. de conf. litt. visit. d. mon. in Ottenbeuren p. d. Johannem prep. fact. 30. mai. 78 S 770 21r -23v, m. (Johanni [de Ceretanis] ep. Nucerin. et al. iudicibus et assistentibus 3 abb. d. ord. reg. observ.) V 667 319r -322v</t>
+          <t>Johannes [de Werdenberg] ep. August. || et presidentes o. s. Ben. inter al. referentes quod Udalricus Huser, Wilhelmus Stendlin, Jodocus Stetter, Udalricus Harder, Lucas Lanczherre, Johannes Brey et Bartholomeus Kystner monachi mon. ss. Alexandri et Theodori mart. in Ottenbeuren o. s. Ben. reg. observ. August. dioc. e d. mon. exierunt ac mitram baculum et al. bona asportarunt et vitam vagabundam ducebant quodque d. ep. et Wilhelmus [de Lustenau] abb. d. mon. in Ottenbeuren litig. contra dd. monachos coram Udalrico [RÃ¶sch] abb. mon. s. Galli de Sancto Gallo Constant. dioc. et coram quond. Johanne de Cesarinis aud. quodque d. ep. d. Wilhelmum propter delapidationem bonorum et al. excessus aliquamdiu suspendit quodque causa abbatibus d. mon. s. Galli et mon. in Salmansweiler Constant. dioc. et deinde Johanni [de Ceretanis] ep. Nucerin. aud. locumtenenti et deinde Johanni Francisco de Pavinis aud. et postremo magistro Johanni de Duchis prep. eccl. Brixien. utr. iur. doct. pape not. commissa fuit: motu pr. de conf. litt. visit. d. mon. in Ottenbeuren p. d. Johannem prep. fact. 30. mai. 78 S 770 21r -23v, m. (Johanni [de Ceretanis] ep. Nucerin. et al. iudicibus et assistentibus 3 abb. d. ord. reg. observ.) V 667 319r -322v</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Johannes vide Joh. Amuelde abb. mon. s. Gregorii in Petridomo e. m. Constant. o. s. Ben. | oblig. p. Johannem Keller can. eccl. s. Johannis Constant. 8 iul. 1426 OC 3 157, O 60 165.</t>
+          <t>Johannes vide Joh. Amuelde abb. mon. s. Gregorii in Petridomo e. m. Constant. o. s. Ben. || oblig. p. Johannem Keller can. eccl. s. Johannis Constant. 8 iul. 1426 OC 3 157, O 60 165.</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Mathias Alardi rect. alt. s. Nicolai in par. eccl. de Herle Leod. dioc. | m. conf. prov. fact. ab Henrico Sticher offic. Frederici aep. Colon. perm. causa inter ipsum et Gerardum Mulrepesch de par. eccl. s. Stephani mon. s. Cornelii Inden. o. s. Ben. Colon. dioc. et de capella s. Nicolai in hosp. pauperum d. mon., 18 mart. 1407 L 129 218.</t>
+          <t>Mathias Alardi rect. alt. s. Nicolai in par. eccl. de Herle Leod. dioc. || m. conf. prov. fact. ab Henrico Sticher offic. Frederici aep. Colon. perm. causa inter ipsum et Gerardum Mulrepesch de par. eccl. s. Stephani mon. s. Cornelii Inden. o. s. Ben. Colon. dioc. et de capella s. Nicolai in hosp. pauperum d. mon., 18 mart. 1407 L 129 218.</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Nicolaus Tylusch de Brega cler. Wratislav. | f. gr. de benef. ad coll. commendatoris etc. domus hosp. s. Johannis Jerus. in Olsen vel abbe. etc. mon. in Trebnitz o. Cist. d. dioc. 29 iun. 1402 L 98 194v.</t>
+          <t>Nicolaus Tylusch de Brega cler. Wratislav. || f. gr. de benef. ad coll. commendatoris etc. domus hosp. s. Johannis Jerus. in Olsen vel abbe. etc. mon. in Trebnitz o. Cist. d. dioc. 29 iun. 1402 L 98 194v.</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Sanderus Marteshusen in palat. ap. servitor | prov. super capel. s. Bartholomei sita infra emunitatem eccl. Paderburn. vac. per ob. Henrici Grashof apud cur., n. o. gr. de benef. ad coll. abb. etc. mon. Corbien. o. s. Ben. Paderburn. dioc., disp. super def. nat. 25 iul. 1414 L 180 102v.</t>
+          <t>Sanderus Marteshusen in palat. ap. servitor || prov. super capel. s. Bartholomei sita infra emunitatem eccl. Paderburn. vac. per ob. Henrici Grashof apud cur., n. o. gr. de benef. ad coll. abb. etc. mon. Corbien. o. s. Ben. Paderburn. dioc., disp. super def. nat. 25 iul. 1414 L 180 102v.</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tuicium | Abb. et conv. mon. s. Heriberti Tuicien. o.s. Ben. Colon. dioc. cui quond. Wilhelmus aep. Colon. certas par. eccl. incorporavit sed cuius effectus n. successerat: de incorp. eidem mon. 128 par. eccl. in Unna 16 m. arg. 3. decb. 1466 S 604 146vs.</t>
+          <t>Tuicium || Abb. et conv. mon. s. Heriberti Tuicien. o.s. Ben. Colon. dioc. cui quond. Wilhelmus aep. Colon. certas par. eccl. incorporavit sed cuius effectus n. successerat: de incorp. eidem mon. 128 par. eccl. in Unna 16 m. arg. 3. decb. 1466 S 604 146vs.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Wilhelmus Thielemanni de Hornbaco presb. Meten. dioc. | de benef. ad coll. abb. etc. mon. s. Pirmini Hornbacen. o. s. Ben. S 76 8.</t>
+          <t>Wilhelmus Thielemanni de Hornbaco presb. Meten. dioc. || de benef. ad coll. abb. etc. mon. s. Pirmini Hornbacen. o. s. Ben. S 76 8.</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>[mon. et op.] Sancti Galli [1. pars 3 partium] Abb. et conv. mon. Sancti Galli o. s. Ben. Constant. dioc. cui par. eccl. in Rottis Vallis Drusione Cur. dioc. ad coll. dd. abb. etc. p. Ortliebum [de Brandis] ep. Cur. incorp. fuit | abb. etc. mon. s. Galli de Sancto Gallo R. E. immediate subiecti o. s. Ben. Constant. dioc.: de lic. erigendi off. scolastr. pro uno scolast. sec. vel reg. d. ord. ad instruendam scientiam litt. noviciis et al. religiosis d. mon. et de incorp. d. officio par. eccl. in Gosiw Constant. dioc. (4 m. arg.) 21. iun. 79 S 783 189v , de ref. 27. oct. 80 S 797 131v â€“</t>
+          <t>[mon. et op.] Sancti Galli [1. pars 3 partium] Abb. et conv. mon. Sancti Galli o. s. Ben. Constant. dioc. cui par. eccl. in Rottis Vallis Drusione Cur. dioc. ad coll. dd. abb. etc. p. Ortliebum [de Brandis] ep. Cur. incorp. fuit || abb. etc. mon. s. Galli de Sancto Gallo R. E. immediate subiecti o. s. Ben. Constant. dioc.: de lic. erigendi off. scolastr. pro uno scolast. sec. vel reg. d. ord. ad instruendam scientiam litt. noviciis et al. religiosis d. mon. et de incorp. d. officio par. eccl. in Gosiw Constant. dioc. (4 m. arg.) 21. iun. 79 S 783 189v , de ref. 27. oct. 80 S 797 131v â€“</t>
         </is>
       </c>
     </row>

</xml_diff>